<commit_message>
Combined scan results 2026-09-26
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,21 +445,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ALAB</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>ABSI</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
@@ -467,18 +475,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANIP</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BAND</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -491,13 +499,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>ADPT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -505,18 +513,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BLFS</t>
+          <t>AEHR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>CHEF</t>
         </is>
       </c>
     </row>
@@ -524,18 +532,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>CAMT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>AKAM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>CRSR</t>
         </is>
       </c>
     </row>
@@ -543,18 +551,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ESLT</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -562,18 +570,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>CORZ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>ALNT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ARW</t>
+          <t>ETON</t>
         </is>
       </c>
     </row>
@@ -581,18 +589,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -600,18 +608,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>ESLT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>FEIM</t>
         </is>
       </c>
     </row>
@@ -619,18 +627,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>ARW</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>COHU</t>
+          <t>FFIV</t>
         </is>
       </c>
     </row>
@@ -638,18 +646,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RGTI</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>AVT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>FTNT</t>
         </is>
       </c>
     </row>
@@ -657,18 +665,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>AXTI</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>GH</t>
         </is>
       </c>
     </row>
@@ -676,153 +684,189 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>LUNR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>BAND</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>GOOGL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>BATRK</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>BLFS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>IBRX</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ORLY</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>BRKR</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>KEEL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>POET</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>META</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>POWL</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>COHU</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>MSFT</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RGTI</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NNBR</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>NESR</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>KOPN</t>
+          <t>OKTA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>STRL</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>OMER</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TLSA</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>DGII</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>PANW</t>
         </is>
       </c>
     </row>
@@ -831,13 +875,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>DIOD</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>PGEN</t>
         </is>
       </c>
     </row>
@@ -846,13 +890,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>DXPE</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MXL</t>
+          <t>PRTH</t>
         </is>
       </c>
     </row>
@@ -861,13 +905,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
@@ -876,13 +920,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>SMTC</t>
         </is>
       </c>
     </row>
@@ -891,13 +935,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
@@ -906,97 +950,73 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>RIOT</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PLXS</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>RXT</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PRTH</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>SIMO</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>KOPN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>TEM</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>TER</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SANM</t>
+          <t>LTRX</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1007,7 +1027,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1018,7 +1038,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SONO</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1029,7 +1049,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1040,7 +1060,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1051,7 +1071,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>VICR</t>
+          <t>MTSI</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1062,11 +1082,330 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>XMTR</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MXL</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NDSN</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>NNBR</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>NTAP</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ORIC</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PLPC</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>PLXS</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>QMCO</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SANM</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SATL</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SIMO</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SITM</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SONO</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SRZN</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>TGTX</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>VICR</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1079,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1107,64 +1446,146 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>AMD</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>CIFR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>AKAM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>HOOD</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GRML</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MARA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GLND</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>MRNA</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
         <is>
           <t>SKHY</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NBIS</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RIOT</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-11
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>BSBR</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>CRDO</t>
         </is>
       </c>
     </row>
@@ -541,13 +541,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BSBR</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>ENTG</t>
         </is>
       </c>
     </row>
@@ -560,13 +560,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EXTR</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -604,7 +604,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -642,7 +642,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -661,7 +661,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -680,7 +680,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>LITE</t>
         </is>
       </c>
     </row>
@@ -688,12 +688,12 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -705,10 +705,14 @@
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -720,7 +724,11 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>CVSA</t>
@@ -729,7 +737,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NNBR</t>
+          <t>P</t>
         </is>
       </c>
     </row>
@@ -738,13 +746,13 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>PANW</t>
         </is>
       </c>
     </row>
@@ -753,13 +761,13 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>RXT</t>
         </is>
       </c>
     </row>
@@ -768,13 +776,13 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>DSP</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
@@ -783,13 +791,13 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>STLN</t>
         </is>
       </c>
     </row>
@@ -798,13 +806,13 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>SYNA</t>
         </is>
       </c>
     </row>
@@ -813,13 +821,13 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RXT</t>
+          <t>VCTR</t>
         </is>
       </c>
     </row>
@@ -828,82 +836,62 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>SYNA</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>VCTR</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>XMTR</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -914,7 +902,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -925,7 +913,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -936,7 +924,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>GSAT</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -947,7 +935,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -958,7 +946,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -969,7 +957,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -980,7 +968,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -991,7 +979,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1002,7 +990,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1013,7 +1001,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1024,7 +1012,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>MGNI</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1035,7 +1023,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1046,7 +1034,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1057,7 +1045,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PNTG</t>
+          <t>NTNX</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1068,7 +1056,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1079,7 +1067,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1090,7 +1078,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>RELL</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1101,7 +1089,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>RZLT</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1112,7 +1100,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1123,7 +1111,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SKWD</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1134,7 +1122,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1145,11 +1133,88 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>RELL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>RZLT</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SKWD</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>XMTR</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1162,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1195,167 +1260,337 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>STNE</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ACHC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>AMPL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>FLEX</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>BWIN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IOVA</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>AVTR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INTR</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>AZTA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NVAX</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NVAX</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>FRSH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>OLB</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>MRNA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VYLR</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>GMAB</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>NTSK</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PENG</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MAT</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>OPCH</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>RXRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>KOD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>STNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NTAP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>SHOP</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>QTEX</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SUNB</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SHLS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>VYLR</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MDLN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-12
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -1585,7 +1585,11 @@
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BTSG</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>NTRA</t>

</xml_diff>

<commit_message>
Combined scan results 2026-10-13
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,7 +447,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,19 +463,15 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>FHB</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ANIP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -486,19 +482,15 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BSBR</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>IDXX</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -509,7 +501,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>BSBR</t>
         </is>
       </c>
     </row>
@@ -517,7 +509,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -528,7 +520,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
@@ -536,7 +528,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -547,7 +539,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>CDNS</t>
         </is>
       </c>
     </row>
@@ -555,18 +547,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FELE</t>
+          <t>ENSG</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>CGNX</t>
         </is>
       </c>
     </row>
@@ -574,18 +566,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FUTU</t>
+          <t>ERIC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>CORT</t>
         </is>
       </c>
     </row>
@@ -593,18 +585,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>CSCO</t>
         </is>
       </c>
     </row>
@@ -612,18 +604,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
@@ -631,18 +623,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>FELE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>EXTR</t>
         </is>
       </c>
     </row>
@@ -650,18 +642,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>FUTU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>FFIV</t>
         </is>
       </c>
     </row>
@@ -669,18 +661,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>FLEX</t>
         </is>
       </c>
     </row>
@@ -688,18 +680,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>FTNT</t>
         </is>
       </c>
     </row>
@@ -707,7 +699,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -718,7 +710,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MTSI</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
@@ -726,216 +718,284 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>IBRX</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LNT</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>IDCC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LSTR</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RXT</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ODFL</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ORLY</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>VCTR</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>NTAP</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>NWE</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>JOYY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -946,7 +1006,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -957,7 +1017,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -968,7 +1028,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>NDSN</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -979,7 +1039,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -990,7 +1050,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1001,7 +1061,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1012,7 +1072,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1023,7 +1083,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1034,7 +1094,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>RELL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1045,7 +1105,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>RZLT</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1056,7 +1116,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1067,7 +1127,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1078,7 +1138,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>SKWD</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1089,7 +1149,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1100,7 +1160,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>STGW</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1111,7 +1171,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1122,99 +1182,11 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>PRCH</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>QLYS</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>RELL</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>RZLT</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>SKWD</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>XMTR</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1227,7 +1199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1255,346 +1227,152 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>ECHO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ACHC</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>OPCH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>GOOGL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>MAT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>VYLR</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>PTC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>FRSH</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NVAX</t>
+          <t>SUNB</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>NTSK</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>TECH</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FTNT</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>MRNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>GMAB</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>IOVA</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GOOGL</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>NTSK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>GOOG</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MAT</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>ISRG</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>OPCH</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>RXRX</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>KOD</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>NTNX</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>STNE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>NTAP</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>OKTA</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>QTEX</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>GTLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PCVX</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>TRMB</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>SUNB</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>ILMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SHLS</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>VYLR</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MDLN</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SNPS</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>BTSG</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>NTRA</t>
-        </is>
-      </c>
+          <t>AFRM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-15
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,7 +447,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,14 +463,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>AMZN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>SUPN</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -486,7 +486,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
@@ -499,13 +499,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BSBR</t>
+          <t>CSCO</t>
         </is>
       </c>
     </row>
@@ -513,12 +513,12 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ALLT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -532,12 +532,12 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>ENSG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -551,7 +551,7 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>ERIC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -562,7 +562,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EZPW</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -581,7 +581,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
@@ -589,18 +589,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FELE</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -613,13 +613,13 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
@@ -627,18 +627,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
@@ -646,18 +646,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
@@ -665,18 +665,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>ODFL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
@@ -684,18 +684,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RZLT</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -703,18 +703,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CLMT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>PCVX</t>
         </is>
       </c>
     </row>
@@ -722,18 +722,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
@@ -741,72 +741,76 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CLWT</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SUPN</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -817,7 +821,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -828,7 +832,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -839,7 +843,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -850,7 +854,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -861,7 +865,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -872,7 +876,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -883,7 +887,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -894,7 +898,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -905,7 +909,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -916,7 +920,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -927,7 +931,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -938,7 +942,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -949,7 +953,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -960,7 +964,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -971,7 +975,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -982,7 +986,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -993,7 +997,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1004,7 +1008,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1015,7 +1019,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1026,7 +1030,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1037,7 +1041,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1048,7 +1052,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1059,7 +1063,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1114,22 +1118,11 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1142,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1170,7 +1163,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1178,118 +1171,26 @@
           <t>AAPL</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
         <is>
           <t>GOOG</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>GOOGL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BORR</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GTLB</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>IBRX</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>SUNB</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>LYFT</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>OPCH</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>MRNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>PYPL</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PENG</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>INTR</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+          <t>BMBL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-16
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,14 +463,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SUPN</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -499,13 +499,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>CHEF</t>
         </is>
       </c>
     </row>
@@ -518,13 +518,13 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>CLOV</t>
         </is>
       </c>
     </row>
@@ -537,13 +537,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
@@ -556,13 +556,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -575,13 +575,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
@@ -594,13 +594,13 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
@@ -608,18 +608,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FUTU</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
@@ -627,18 +627,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -646,18 +646,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -670,13 +670,13 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>PCVX</t>
         </is>
       </c>
     </row>
@@ -689,13 +689,13 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
@@ -708,13 +708,13 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -722,18 +722,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
@@ -741,37 +741,33 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CLWT</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>SHOP</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
@@ -780,37 +776,29 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>STLD</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -821,7 +809,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -832,7 +820,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>EZPW</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -843,7 +831,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -854,7 +842,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -865,7 +853,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -876,7 +864,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -887,7 +875,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -898,7 +886,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -909,7 +897,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -920,7 +908,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -931,7 +919,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -942,7 +930,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -953,7 +941,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -964,7 +952,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -975,7 +963,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -986,7 +974,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -997,7 +985,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1008,7 +996,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1019,110 +1007,11 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>NSIT</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>OPLN</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1163,32 +1052,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GOOGL</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
           <t>AAPL</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>GOOG</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MRNA</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BMBL</t>
-        </is>
-      </c>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Combined scan results 2026-10-17
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,7 +447,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -457,25 +457,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ATAT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -486,26 +486,30 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>CLMT</t>
         </is>
       </c>
     </row>
@@ -513,18 +517,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>CASY</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AFRM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
@@ -532,18 +536,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -551,18 +555,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -575,13 +579,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
@@ -594,13 +598,13 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>MSFT</t>
         </is>
       </c>
     </row>
@@ -608,18 +612,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -627,18 +631,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>ONC</t>
         </is>
       </c>
     </row>
@@ -646,12 +650,12 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -665,18 +669,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
@@ -684,18 +688,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>ODFL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -708,13 +712,13 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>SHOP</t>
         </is>
       </c>
     </row>
@@ -722,18 +726,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CHEF</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>STLD</t>
         </is>
       </c>
     </row>
@@ -741,42 +745,38 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VMRK</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -787,7 +787,7 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -798,7 +798,7 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -809,7 +809,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -820,7 +820,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -831,7 +831,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -842,7 +842,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -853,7 +853,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>ECPG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -864,7 +864,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -875,7 +875,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -886,7 +886,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>EZPW</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -897,7 +897,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -908,7 +908,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -919,7 +919,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -930,7 +930,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -941,7 +941,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -952,7 +952,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -963,7 +963,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -974,7 +974,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -985,7 +985,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -996,7 +996,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1007,11 +1007,154 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MTCH</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SHOO</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1024,7 +1167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1055,19 +1198,443 @@
           <t>AAPL</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PDD</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BORR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PTON</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DBX</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ARQT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AEP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FRSH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ASO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GMAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GEHC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BIIB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CAKE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>INTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BSY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MDLN</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>LIFE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CCEP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MTCH</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CME</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>COR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>OPCH</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CTAS</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DOCU</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NVAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EXEL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EXLS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>VYLR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>HTHT</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>WLTH</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>KDP</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>LAUR</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NAVN</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>NTAP</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OLLI</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OTEX</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>STRC</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ACHC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-18
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,12 +452,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ATAT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -470,23 +470,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATAT</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
@@ -498,18 +498,18 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>CASY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
@@ -517,18 +517,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>CDZI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -541,13 +541,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
@@ -560,13 +560,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ALLT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
@@ -574,18 +574,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>ESLT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -593,18 +593,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ECPG</t>
         </is>
       </c>
     </row>
@@ -612,18 +612,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -631,18 +631,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -650,18 +650,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
@@ -669,18 +669,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BCPC</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>MTCH</t>
         </is>
       </c>
     </row>
@@ -693,13 +693,13 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -737,7 +737,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -754,7 +754,11 @@
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SHOO</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
@@ -769,7 +773,11 @@
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
@@ -780,7 +788,11 @@
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
@@ -791,7 +803,11 @@
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
@@ -820,7 +836,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -831,7 +847,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -842,7 +858,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -853,7 +869,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ECPG</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -864,7 +880,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -875,7 +891,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -886,7 +902,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -897,7 +913,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -908,7 +924,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -919,7 +935,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -930,7 +946,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -941,7 +957,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -952,7 +968,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -963,7 +979,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -974,7 +990,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -985,7 +1001,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -996,7 +1012,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1007,7 +1023,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1018,7 +1034,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1029,132 +1045,11 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>NWSA</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>PLMR</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>SHOO</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1167,7 +1062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1200,61 +1095,61 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ACHC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PDD</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>EXC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BORR</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PTON</t>
+          <t>LIFE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>MRSH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
@@ -1266,375 +1161,261 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>AVTR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GEHC</t>
+          <t>BZ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>TCRT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>CSGP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>BORR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MDLN</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CCC</t>
-        </is>
-      </c>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MRNA</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CDW</t>
-        </is>
-      </c>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MTCH</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CME</t>
-        </is>
-      </c>
+          <t>CTAS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>MDLZ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>GEHC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OPCH</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CTAS</t>
-        </is>
-      </c>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>NAVN</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PYPL</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>DOCU</t>
-        </is>
-      </c>
+          <t>FANG</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NVAX</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TECH</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>EXEL</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>VYLR</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TRMB</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>EXLS</t>
-        </is>
-      </c>
+          <t>KDP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>OLLI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VYLR</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>GTLB</t>
-        </is>
-      </c>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>HTHT</t>
-        </is>
-      </c>
+          <t>NCPL</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WLTH</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>ISRG</t>
-        </is>
-      </c>
+          <t>TECH</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>KDP</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>LAUR</t>
-        </is>
-      </c>
+          <t>BMBL</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>LYFT</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MDLZ</t>
+          <t>OTEX</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>NAVN</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>NTAP</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>OLLI</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>OTEX</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>STRC</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ACHC</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-20
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,9 +414,810 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>1. 信號反轉-底背離</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2. 信號反轉-回升</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>3. 機會入場</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>4. 重新起漲</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>5. 空中加油</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ATAT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ATMU</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ACGL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AUPH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AZN</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ACIW</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>BIIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CASY</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>COLB</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AER</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>COR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DORM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AGYS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ESLT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ALLT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DBX</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FHB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GPGI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ECPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>EVRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LSTR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ARQT</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>GCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NXST</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ASO</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>OSIS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>AVPT</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>GSAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OZK</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BCPC</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>HURN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CAKE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LAUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CCEP</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LGND</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CHEF</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CHRD</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VMRK</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CINF</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>OPLN</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CME</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>POWW</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>COKE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SHOO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CVSA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DAVE</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>EXEL</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FANG</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FTDR</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GMAB</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>HALO</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>HTHT</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KDP</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEDP</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MEOH</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MTCH</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -427,9 +1228,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>強勢+站穩+大量</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>開漲+站穩</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>開漲+大量</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>開漲</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EXE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GMAB</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>KDP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ARQT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CSX</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TCRT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Combined scan results 2026-10-21
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ATAT</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -459,7 +459,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -478,7 +478,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -497,7 +497,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -516,7 +516,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
@@ -524,18 +524,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -543,18 +543,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -562,18 +562,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ESLT</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -581,18 +581,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
@@ -600,18 +600,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ECPG</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
@@ -619,18 +619,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -638,18 +638,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BCPC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -657,220 +657,156 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>OSIS</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>SHOO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>OZK</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PECO</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>LAUR</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>PNFP</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>LGND</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>NTES</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>NWSA</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>OPLN</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>POWW</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>SHOO</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -881,7 +817,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -892,7 +828,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -903,7 +839,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -914,7 +850,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -925,7 +861,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -947,7 +883,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -958,7 +894,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -969,7 +905,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -980,7 +916,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -991,7 +927,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1002,7 +938,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1013,7 +949,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1024,7 +960,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1035,7 +971,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1046,7 +982,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1057,7 +993,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1068,7 +1004,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1079,7 +1015,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1090,7 +1026,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1101,7 +1037,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1112,7 +1048,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1123,7 +1059,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1134,7 +1070,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1145,7 +1081,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1156,7 +1092,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1167,7 +1103,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1178,7 +1114,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1189,7 +1125,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1200,7 +1136,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1211,11 +1147,110 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1228,7 +1263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1256,100 +1291,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EXE</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>GMAB</t>
-        </is>
-      </c>
+          <t>BRZE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>APA</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>FAST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>KDP</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>ARQT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CSX</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
           <t>HAS</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>LYFT</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ISRG</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MNST</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TCRT</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CTSH</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-22
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -459,7 +459,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
@@ -467,18 +467,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>AFRM</t>
         </is>
       </c>
     </row>
@@ -486,18 +486,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
@@ -505,18 +505,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>CRMD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -535,7 +535,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
@@ -543,18 +543,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -562,18 +562,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
@@ -581,18 +581,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
@@ -600,18 +600,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -630,7 +630,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
@@ -638,18 +638,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>MIDD</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>CORT</t>
         </is>
       </c>
     </row>
@@ -657,156 +657,224 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>BTSG</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>OSIS</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SHOO</t>
+          <t>CYRX</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OZK</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>FANG</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GSAT</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>KDP</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LGND</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>VMRK</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -817,7 +885,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -828,7 +896,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -839,7 +907,7 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -861,7 +929,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -872,7 +940,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -883,7 +951,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -894,7 +962,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -905,7 +973,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -916,7 +984,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -927,7 +995,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -938,7 +1006,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -949,7 +1017,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -960,7 +1028,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>JOYY</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -971,7 +1039,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -982,7 +1050,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -993,7 +1061,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1004,7 +1072,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1015,7 +1083,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1026,7 +1094,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1037,7 +1105,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1048,7 +1116,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1059,7 +1127,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1070,7 +1138,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1081,7 +1149,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1092,7 +1160,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1103,7 +1171,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>ORIC</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1114,7 +1182,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1125,7 +1193,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1136,7 +1204,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1147,7 +1215,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1158,7 +1226,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1169,7 +1237,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1180,7 +1248,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1191,7 +1259,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1202,7 +1270,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>SEIC</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1213,7 +1281,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>SEZL</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1224,7 +1292,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1235,7 +1303,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>SLN</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1246,11 +1314,55 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1263,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1289,22 +1401,24 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>BRZE</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
         <is>
           <t>MRNA</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-23
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,21 +445,25 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ABNB</t>
         </is>
       </c>
     </row>
@@ -467,18 +471,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
@@ -486,18 +490,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>CARG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -505,18 +509,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CASH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
@@ -535,7 +539,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -554,7 +558,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
@@ -567,13 +571,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -586,13 +590,13 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
@@ -600,18 +604,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
@@ -619,18 +623,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
@@ -638,18 +642,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MIDD</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
@@ -657,18 +661,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
@@ -676,18 +680,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -695,18 +699,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CRON</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EXPE</t>
         </is>
       </c>
     </row>
@@ -714,12 +718,12 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>RYAAY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -733,18 +737,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>TBLA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>FROG</t>
         </is>
       </c>
     </row>
@@ -752,66 +756,54 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>RYAAY</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CYRX</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>DAVE</t>
@@ -820,7 +812,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
@@ -835,7 +827,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>MNST</t>
         </is>
       </c>
     </row>
@@ -844,13 +836,13 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>DCOM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>NTNX</t>
         </is>
       </c>
     </row>
@@ -859,13 +851,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -874,11 +866,15 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PAYO</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
@@ -889,36 +885,48 @@
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -962,7 +970,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -984,7 +992,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -995,7 +1003,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1028,7 +1036,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1039,7 +1047,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1061,7 +1069,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1072,7 +1080,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1083,7 +1091,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1094,7 +1102,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1105,7 +1113,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1116,7 +1124,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1127,7 +1135,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1138,7 +1146,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1204,7 +1212,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1215,7 +1223,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1226,7 +1234,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1237,7 +1245,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>RELY</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1248,7 +1256,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1259,7 +1267,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1270,7 +1278,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1281,7 +1289,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>SEIC</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1292,7 +1300,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>SEZL</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1303,7 +1311,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1314,7 +1322,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>SLN</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1325,7 +1333,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1336,7 +1344,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TNGX</t>
+          <t>STLN</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1347,7 +1355,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>TNGX</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1358,11 +1366,33 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>UTHR</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1375,7 +1405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1401,24 +1431,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IOVA</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>CSX</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KDP</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>MRNA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-24
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,14 +445,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>ANIP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,7 +467,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,7 +486,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -509,7 +505,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -520,7 +516,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -528,18 +524,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CRMD</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
@@ -547,18 +543,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>BOKF</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>CLOV</t>
         </is>
       </c>
     </row>
@@ -566,18 +562,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>CARG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>CRSR</t>
         </is>
       </c>
     </row>
@@ -585,18 +581,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>CASH</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
@@ -604,18 +600,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>CRMD</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>ASO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -623,18 +619,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
@@ -642,18 +638,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
@@ -661,18 +657,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>IRTC</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>BCPC</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
@@ -680,18 +676,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
@@ -699,18 +695,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>MIDD</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>MTCH</t>
         </is>
       </c>
     </row>
@@ -718,18 +714,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -737,18 +733,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TBLA</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -756,177 +752,161 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>ROST</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>TECH</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TROO</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>KNSA</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>VMRK</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CRON</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>MNST</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>NTNX</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>OPLN</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>PAYO</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>RGEN</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>ROST</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>CYRX</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>DAVE</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -937,7 +917,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -948,7 +928,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>DCOM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -959,7 +939,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -970,7 +950,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -981,7 +961,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -992,7 +972,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1003,7 +983,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1014,7 +994,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1025,7 +1005,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1036,7 +1016,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1047,7 +1027,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1058,7 +1038,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1069,7 +1049,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1080,7 +1060,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1091,7 +1071,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1102,7 +1082,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1113,7 +1093,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1124,7 +1104,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1135,7 +1115,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1146,7 +1126,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1157,7 +1137,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1168,7 +1148,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1179,7 +1159,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1190,7 +1170,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1201,7 +1181,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1212,7 +1192,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1223,7 +1203,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1234,7 +1214,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1245,7 +1225,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1256,7 +1236,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1267,7 +1247,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1278,7 +1258,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1289,7 +1269,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1300,7 +1280,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1311,7 +1291,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1322,7 +1302,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1333,7 +1313,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1344,7 +1324,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>ORIC</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1355,7 +1335,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>TNGX</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1366,7 +1346,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1377,7 +1357,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1388,11 +1368,187 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>PAYO</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1405,7 +1561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1438,15 +1594,427 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>ACGL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>CSX</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PODD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AZN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>HONA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BSP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ODFL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ETSY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AEP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EXEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AMCR</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CME</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AMGN</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EXE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ASO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FRSH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>APPN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BSY</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GEHC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KMB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>IRON</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CCEP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CSGP</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PEGA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CTAS</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DBX</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DOCU</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EXC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EVRG</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EXLS</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FOXA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ORLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LNT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GMAB</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MRSH</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NCNO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
         <is>
           <t>KDP</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>HALO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SGRY</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SUNB</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-25
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LSTR</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>ANIP</t>
@@ -459,7 +463,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
@@ -467,18 +471,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ACIW</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
@@ -486,18 +490,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -505,18 +509,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
@@ -524,18 +528,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>BLBD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CRON</t>
         </is>
       </c>
     </row>
@@ -548,13 +552,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CRSR</t>
         </is>
       </c>
     </row>
@@ -567,13 +571,13 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>APPN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CRSR</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -592,7 +596,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
@@ -605,13 +609,13 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
@@ -619,7 +623,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -630,7 +634,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -638,7 +642,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -649,7 +653,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -657,7 +661,7 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -668,7 +672,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>EXPE</t>
         </is>
       </c>
     </row>
@@ -676,7 +680,7 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -687,7 +691,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>FOX</t>
         </is>
       </c>
     </row>
@@ -695,7 +699,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MIDD</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -706,7 +710,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>FOXA</t>
         </is>
       </c>
     </row>
@@ -714,7 +718,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -725,7 +729,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>FTNT</t>
         </is>
       </c>
     </row>
@@ -733,18 +737,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CENTA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
@@ -752,18 +756,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -776,13 +780,13 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
@@ -790,222 +794,282 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>TROO</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>VMRK</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LLYVK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LOGI</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MTCH</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>DLO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>OPLN</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ORIC</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PAYO</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1016,7 +1080,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1027,7 +1091,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1038,7 +1102,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1049,7 +1113,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1060,7 +1124,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1071,7 +1135,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1082,7 +1146,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1093,7 +1157,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1104,7 +1168,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1115,7 +1179,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1126,7 +1190,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1137,7 +1201,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1148,7 +1212,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1159,7 +1223,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>NWBI</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1170,7 +1234,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1181,7 +1245,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1192,7 +1256,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1203,7 +1267,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1214,7 +1278,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1225,7 +1289,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1236,7 +1300,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1247,7 +1311,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>QLYS</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1258,7 +1322,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1269,7 +1333,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1280,7 +1344,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1291,7 +1355,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>SFNC</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1302,7 +1366,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1313,7 +1377,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>UTHR</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1324,7 +1388,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1335,220 +1399,11 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>XNCR</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>PAGP</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>PAYO</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>PLMR</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>QLYS</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>REGN</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>ROKU</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>RPRX</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>SIGI</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr"/>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr"/>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>TNGX</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr"/>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr"/>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr"/>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1589,34 +1444,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>AMPL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>AVTR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>CELH</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>BRZE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1626,36 +1481,36 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>NXPI</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>APPN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BSP</t>
+          <t>BSY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1665,339 +1520,319 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>SBAC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>SOLS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>BZ</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>DOCU</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>CTAS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>EXE</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ASO</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>GMAB</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GEHC</t>
+          <t>INTR</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>ERIC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>FRSH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>NTSK</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>IOVA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CSGP</t>
+          <t>GEHC</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PEGA</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>IRON</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>HTFL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>CSGP</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>NAVN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>LIFE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>AMCR</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>KMB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EVRG</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
+          <t>MTCH</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>TRI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EXLS</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>NDAQ</t>
-        </is>
-      </c>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>FISV</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>FOXA</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>ORLY</t>
-        </is>
-      </c>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LNT</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GMAB</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MRSH</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>HAS</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>SSNC</t>
-        </is>
-      </c>
+          <t>CME</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NCNO</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>INTU</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>TRMB</t>
-        </is>
-      </c>
+          <t>MRSH</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KDP</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>HALO</t>
-        </is>
-      </c>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SGRY</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -2005,15 +1840,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>EXLS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MDLZ</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Combined scan results 2026-10-26
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -1515,7 +1515,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CHKP</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>INTR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>CDW</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>TENB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>ERIC</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>AMCR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>HCSG</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CSGP</t>
+          <t>HTFL</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>ISRG</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1721,7 +1721,11 @@
           <t>MTCH</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1729,17 +1733,17 @@
           <t>SHOP</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>TRI</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>PTC</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1747,17 +1751,17 @@
           <t>TEAM</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>FISV</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1765,17 +1769,17 @@
           <t>TW</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ADP</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TENB</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>SLDE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1783,14 +1787,10 @@
           <t>VSXY</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>TRI</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1798,13 +1798,13 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>EXLS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MRSH</t>
+          <t>KMB</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1812,13 +1812,13 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1826,13 +1826,13 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>SLN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>CSGP</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1840,7 +1840,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>MRSH</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-27
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,31 +447,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ANIP</t>
+          <t>AMBA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LSTR</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>ANIP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -482,7 +486,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ADI</t>
         </is>
       </c>
     </row>
@@ -490,18 +494,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
@@ -520,7 +524,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
@@ -539,7 +543,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -558,7 +562,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CRSR</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -577,7 +581,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -585,7 +589,7 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -596,7 +600,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
@@ -604,18 +608,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRMD</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -623,7 +627,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -634,7 +638,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -642,7 +646,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -661,18 +665,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>FFIV</t>
         </is>
       </c>
     </row>
@@ -680,12 +684,12 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -699,12 +703,12 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>PATK</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -718,12 +722,12 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>RYAAY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>CENTA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -737,75 +741,63 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>TPG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>OSIS</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>LIVN</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>TPG</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
@@ -814,13 +806,13 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>MNST</t>
         </is>
       </c>
     </row>
@@ -829,13 +821,13 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -850,7 +842,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>NTNX</t>
         </is>
       </c>
     </row>
@@ -865,7 +857,7 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>NWS</t>
         </is>
       </c>
     </row>
@@ -880,7 +872,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>NWSA</t>
         </is>
       </c>
     </row>
@@ -895,7 +887,7 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
@@ -910,7 +902,7 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
@@ -925,7 +917,7 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
@@ -934,13 +926,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -949,13 +941,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>ROKU</t>
         </is>
       </c>
     </row>
@@ -964,13 +956,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
@@ -979,13 +971,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PAYO</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
@@ -994,13 +986,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>SRZN</t>
         </is>
       </c>
     </row>
@@ -1009,13 +1001,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
@@ -1024,52 +1016,40 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>FFBC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>FITB</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1080,7 +1060,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1091,7 +1071,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1102,7 +1082,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>FULT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1113,7 +1093,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1124,7 +1104,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1135,7 +1115,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1146,7 +1126,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1157,7 +1137,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1168,7 +1148,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1179,7 +1159,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1190,7 +1170,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1201,7 +1181,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1212,7 +1192,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1223,7 +1203,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1234,7 +1214,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1245,7 +1225,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1256,7 +1236,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1267,7 +1247,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1278,7 +1258,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1289,7 +1269,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1300,7 +1280,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>NMIH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1311,7 +1291,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1322,7 +1302,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>NWBI</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1333,7 +1313,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1344,7 +1324,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1355,7 +1335,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1366,7 +1346,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1377,7 +1357,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1388,7 +1368,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>PAYO</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1399,11 +1379,165 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SBCF</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1416,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1444,408 +1578,82 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>NTSK</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>SGRY</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>NXPI</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ASST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>HONA</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>TNGX</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>APPN</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BSY</t>
-        </is>
-      </c>
+          <t>ERIC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>PEGA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CHKP</t>
-        </is>
-      </c>
+          <t>GMAB</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SBAC</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SOLS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>BZ</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GMAB</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DOCU</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CART</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>EBAY</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>INTR</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>EXE</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CDW</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>GTLB</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>NTSK</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>FANG</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>CTAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>HALO</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>FRSH</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>DBX</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>IOVA</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>GEHC</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ERIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>IRON</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>AMCR</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>HCSG</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PAYX</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>HTFL</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>NAVN</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CME</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>LIFE</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ISRG</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>NRIX</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>CTSH</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>MTCH</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>PAGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>SHOP</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>PTC</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>RPRX</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>RELY</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>FISV</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TW</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>SLDE</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>INTU</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>TRI</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>EXLS</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>KMB</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ADP</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>CSGP</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>MRSH</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+          <t>BRZE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Combined scan results 2026-10-28
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,11 +445,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>BKR</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>AMBA</t>
@@ -457,30 +453,26 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ACT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LSTR</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANIP</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -494,18 +486,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
@@ -518,7 +510,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -537,13 +529,13 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -556,13 +548,13 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -570,18 +562,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>CALY</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
@@ -589,18 +581,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -608,18 +600,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BUSE</t>
         </is>
       </c>
     </row>
@@ -627,18 +619,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CFR</t>
         </is>
       </c>
     </row>
@@ -646,18 +638,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CENTA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -665,18 +657,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>EXTR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>CGNT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
@@ -684,18 +676,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
@@ -703,18 +695,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
@@ -722,18 +714,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
@@ -741,93 +733,113 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NXST</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>OSIS</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>FANG</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PATK</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>FITB</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>FFIV</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
@@ -836,13 +848,13 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>FULT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>FTNT</t>
         </is>
       </c>
     </row>
@@ -851,13 +863,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
@@ -866,13 +878,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
@@ -881,13 +893,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>HCSG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
@@ -896,13 +908,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -911,13 +923,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
@@ -926,13 +938,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -941,13 +953,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>ICUI</t>
         </is>
       </c>
     </row>
@@ -956,13 +968,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
@@ -971,13 +983,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>LIVN</t>
         </is>
       </c>
     </row>
@@ -986,13 +998,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>NMIH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
@@ -1001,13 +1013,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>NSIT</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -1016,528 +1028,191 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>NUTX</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NWBI</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>QLYS</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>SFNC</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>SIGI</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>SRZN</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>SYRE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>XNCR</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>HQY</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>HTHT</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>HURN</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>ICUI</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>INDB</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>LFST</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>LIN</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>LOGI</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>MEDP</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>MEOH</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>NDAQ</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>NMIH</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>NSIT</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr"/>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>NWBI</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>NWE</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>OSPN</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr"/>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>OZK</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr"/>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr"/>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>PAGP</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>PAYO</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr"/>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>PNFP</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>PTEN</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>QLYS</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>ROST</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>RPRX</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>SBCF</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>SFNC</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>SIGI</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>SWIM</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>SYRE</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1550,7 +1225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1578,80 +1253,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>BRZE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SGRY</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NXPI</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ASST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GILD</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>TNGX</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ERIC</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PEGA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>GTLB</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
           <t>GMAB</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>PYPL</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>BRZE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Combined scan results 2026-10-29
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ENSG</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>AMBA</t>
@@ -453,13 +457,13 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>ABCL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
@@ -467,18 +471,18 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ABSI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -486,18 +490,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
@@ -510,13 +514,13 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -524,18 +528,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BLBD</t>
+          <t>BOKF</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>ADPT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
@@ -543,18 +547,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BOKF</t>
+          <t>CALY</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>CFR</t>
         </is>
       </c>
     </row>
@@ -562,18 +566,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CALY</t>
+          <t>CARG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
@@ -581,18 +585,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>CERS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
@@ -600,18 +604,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUSE</t>
+          <t>EBC</t>
         </is>
       </c>
     </row>
@@ -619,18 +623,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>CRML</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -638,18 +642,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
@@ -657,18 +661,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
@@ -676,18 +680,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>BBT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
@@ -695,18 +699,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>ESTA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>BOW</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>GLBE</t>
         </is>
       </c>
     </row>
@@ -714,18 +718,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>BRKR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -733,18 +737,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -752,18 +756,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
@@ -771,18 +775,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>CGNT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>NMIH</t>
         </is>
       </c>
     </row>
@@ -790,18 +794,18 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>OCFC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
@@ -809,18 +813,18 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>OSIS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>OZK</t>
         </is>
       </c>
     </row>
@@ -828,48 +832,56 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>PATK</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>STOK</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>ESQ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>PNFP</t>
         </is>
       </c>
     </row>
@@ -878,13 +890,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
@@ -893,13 +905,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>SFNC</t>
         </is>
       </c>
     </row>
@@ -908,13 +920,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
@@ -923,13 +935,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>FCNCA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>STLN</t>
         </is>
       </c>
     </row>
@@ -938,13 +950,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>TCBK</t>
         </is>
       </c>
     </row>
@@ -953,13 +965,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>TECH</t>
         </is>
       </c>
     </row>
@@ -968,13 +980,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
@@ -983,13 +995,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
@@ -998,221 +1010,484 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>LOGI</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>NRIX</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>NTNX</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>GSAT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>NUTX</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>NWBI</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>PAA</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>PAGP</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>PNFP</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>KYMR</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>REGN</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>SLAB</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>SLN</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SYRE</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>TECH</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NBN</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>NOVT</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NUTX</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NWE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>OSW</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>PTEN</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>RDNT</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>RDWR</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TGTX</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1225,7 +1500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1253,22 +1528,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ETSY</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>GMAB</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EXC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GEHC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>CSX</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>GMAB</t>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FITB</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SBUX</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Combined scan results 2026-10-30
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,23 +452,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AMBA</t>
+          <t>AAL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FWONK</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>ATMU</t>
@@ -476,13 +480,13 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>ABCL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AFRM</t>
         </is>
       </c>
     </row>
@@ -490,18 +494,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ABSI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>AMCR</t>
         </is>
       </c>
     </row>
@@ -509,18 +513,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>BLBD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
@@ -528,18 +532,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BOKF</t>
+          <t>CALY</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ADPT</t>
+          <t>ACT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -547,18 +551,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CALY</t>
+          <t>CERS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
@@ -566,18 +570,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ADPT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
@@ -585,18 +589,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CERS</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ADUS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
@@ -604,18 +608,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -623,18 +627,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CRML</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>ALKS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
@@ -642,18 +646,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>DRS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
@@ -661,18 +665,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>ELDN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
@@ -680,18 +684,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>ESTA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -699,18 +703,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ESTA</t>
+          <t>EVLV</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
@@ -718,18 +722,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>FER</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BRKR</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>FANG</t>
         </is>
       </c>
     </row>
@@ -737,18 +741,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AXGN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
@@ -756,18 +760,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>BOW</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>FSUN</t>
         </is>
       </c>
     </row>
@@ -775,18 +779,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>INDV</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>BRKR</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
@@ -794,18 +798,18 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>OCFC</t>
+          <t>NBIX</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CATY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -813,18 +817,18 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>NEXT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>CFR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>MDB</t>
         </is>
       </c>
     </row>
@@ -832,18 +836,18 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>NDSN</t>
         </is>
       </c>
     </row>
@@ -851,18 +855,18 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>STOK</t>
+          <t>OCFC</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
@@ -870,108 +874,132 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>PTCT</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>STOK</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>DORM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>EBC</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TBLA</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>TCBK</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>ESQ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
@@ -980,13 +1008,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>SBCF</t>
         </is>
       </c>
     </row>
@@ -995,13 +1023,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
@@ -1010,62 +1038,82 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>FFBC</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>FIBK</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>FITB</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1076,7 +1124,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1087,7 +1135,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>FULT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1098,7 +1146,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KYMR</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1109,7 +1157,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1120,7 +1168,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>GLBE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1131,7 +1179,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1142,7 +1190,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1153,7 +1201,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1164,7 +1212,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1175,7 +1223,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NBN</t>
+          <t>ICUI</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1186,7 +1234,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>INDB</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1197,7 +1245,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1208,7 +1256,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>KYMR</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1219,7 +1267,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1230,7 +1278,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NUTX</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1241,7 +1289,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1252,7 +1300,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1263,7 +1311,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1274,7 +1322,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1285,7 +1333,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ORKA</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1296,7 +1344,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>MGRC</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1307,7 +1355,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>NBN</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1318,7 +1366,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1329,7 +1377,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>NMIH</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1340,7 +1388,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>RDNT</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1351,7 +1399,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>RDWR</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1362,7 +1410,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>NTRA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1373,7 +1421,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>OABI</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1384,7 +1432,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>RLAY</t>
+          <t>ORKA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1395,7 +1443,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1406,7 +1454,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1417,7 +1465,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SGMT</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1428,7 +1476,7 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -1439,7 +1487,7 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SYRE</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -1450,7 +1498,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TGTX</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -1461,7 +1509,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>VISN</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -1472,7 +1520,7 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>RDNT</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -1483,11 +1531,253 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>RDWR</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>REPL</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>RGEN</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SHC</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>STGW</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr"/>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>TCBK</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>TGTX</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>VCTR</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr"/>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1500,7 +1790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1533,29 +1823,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>CPRT</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>MFIC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1565,25 +1855,73 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GEHC</t>
+          <t>SIRI</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HBAN</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>CSX</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>FITB</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>SBUX</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>KDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AIOK</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GEHC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SGRY</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PGY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Combined scan results 2026-10-31
</commit_message>
<xml_diff>
--- a/results/latest.xlsx
+++ b/results/latest.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,11 +445,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ENSG</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>AAL</t>
@@ -463,30 +459,26 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ABSI</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>FWONK</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATMU</t>
+          <t>BCRX</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>ACGL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
@@ -494,18 +486,18 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>ADPT</t>
         </is>
       </c>
     </row>
@@ -513,18 +505,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BLBD</t>
+          <t>BKU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ADUS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -532,18 +524,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CALY</t>
+          <t>BOKF</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
@@ -551,18 +543,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CERS</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>AER</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -570,18 +562,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ADPT</t>
+          <t>ALKS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
@@ -589,18 +581,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CRSP</t>
+          <t>DRS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AMCR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
@@ -608,18 +600,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>EVLV</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BBT</t>
         </is>
       </c>
     </row>
@@ -627,18 +619,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>FTAI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
@@ -646,18 +638,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DRS</t>
+          <t>FWONK</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
@@ -665,18 +657,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ELDN</t>
+          <t>INDV</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
@@ -684,18 +676,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ESTA</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>AXGN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
@@ -703,18 +695,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EVLV</t>
+          <t>PODC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>BJRI</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>CFR</t>
         </is>
       </c>
     </row>
@@ -722,18 +714,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FER</t>
+          <t>PTCT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>BTSG</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
@@ -741,18 +733,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>RYAAY</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>CCEP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
@@ -760,18 +752,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>RYTM</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FSUN</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
@@ -779,18 +771,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>INDV</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BRKR</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
@@ -798,18 +790,18 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>STOK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>EBC</t>
         </is>
       </c>
     </row>
@@ -817,18 +809,18 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NEXT</t>
+          <t>SUPN</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>ESQ</t>
         </is>
       </c>
     </row>
@@ -836,18 +828,18 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>SVRA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
@@ -855,66 +847,54 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>OCFC</t>
+          <t>TBLA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CROX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>PTCT</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>RYAAY</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>FIBK</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>SOFI</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>DLTR</t>
@@ -923,17 +903,13 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>STOK</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>DORM</t>
@@ -942,64 +918,52 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>SUPN</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>GH</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>TBLA</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>TPG</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -1008,13 +972,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SBCF</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
@@ -1023,13 +987,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>KYMR</t>
         </is>
       </c>
     </row>
@@ -1038,13 +1002,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>MSGK</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1023,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
@@ -1068,13 +1032,13 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
@@ -1083,13 +1047,13 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -1098,13 +1062,13 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>GEN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>OZK</t>
         </is>
       </c>
     </row>
@@ -1113,227 +1077,307 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>RDNT</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>RDWR</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SBCF</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>LLYVA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TCBK</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>KYMR</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TECH</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>ORKA</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TLS</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>OSPN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>VISN</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PFG</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>PLMR</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1344,7 +1388,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MGRC</t>
+          <t>PNFP</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1355,7 +1399,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>NBN</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1366,7 +1410,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1377,7 +1421,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1388,7 +1432,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>PVLA</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1399,7 +1443,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1410,7 +1454,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>REPL</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1421,7 +1465,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1432,7 +1476,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ORKA</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1443,7 +1487,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>SAIC</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1454,7 +1498,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>STGW</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1465,7 +1509,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1476,7 +1520,7 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -1487,7 +1531,7 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>TGTX</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -1498,7 +1542,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -1509,7 +1553,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>UTHR</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -1520,264 +1564,11 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>RDNT</t>
+          <t>VCTR</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>RDWR</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>REGN</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>REPL</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>RGEN</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>RLAY</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>ROIV</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>SBUX</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr"/>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr"/>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>SFNC</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr"/>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>SGMT</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr"/>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>SHC</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr"/>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>STGW</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr"/>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>STLD</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr"/>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>SYRE</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr"/>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>TCBK</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr"/>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>TEM</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr"/>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr"/>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>TGTX</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr"/>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr"/>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr"/>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>VCTR</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>VISN</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1790,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1818,110 +1609,168 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>HBAN</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>AZN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FISV</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>BBIO</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>MFIC</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>EXC</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>SIRI</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>SIRI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HBAN</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>BSY</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>CPRT</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>EXEL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>EXC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AIOK</t>
+          <t>GEHC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GEHC</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SGRY</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PGY</t>
+          <t>GMAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>KHC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LNT</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GILD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>RXRX</t>
         </is>
       </c>
     </row>

</xml_diff>